<commit_message>
Clue Words: integrate richer source file (55 clues + frequency)
- New source content/sources/clue_workbook.xlsx (Positive 26 + Negative 29),
  replacing the old 39-entry master clue data.
- Carry "matched question count" -> sort clues by exam frequency and show
  "Appears in ~N exam questions" on the lesson card.
- Fuller general-use context + clean watch-out notes (drop EXCEPTION_OVERRIDE).
- Fix stripped Finnish diacritics: 51 verified token repairs in
  content/clue_fi_fixes.json (valita->välitä homograph deliberately blacklisted);
  0 broken phrases remain.
- build_clue.py rewritten for the 2-sheet format + diacritic repair.
- master.xlsx Clue_Words sheet updated to match (55 rows + Source-sets column).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/sources/master.xlsx
+++ b/content/sources/master.xlsx
@@ -505,7 +505,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -659,8 +658,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
@@ -25335,7 +25332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -25402,6 +25399,11 @@
           <t>Bangla — to fill</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Source sets covered</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -25416,35 +25418,38 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>varmistaa / varmistua / huolehtia</t>
+          <t>poliisi / liikenteen valvoja / hätäkeskus</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>make sure / take care</t>
+          <t>police / traffic controller / emergency centre / 112</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive when authority help is needed: accident, threat, unpaid fare, traffic control, or a person who cannot safely be left.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Often correct in safety-duty answers</t>
+          <t>Do not call police for every ordinary customer-service problem; first use calm communication where safe.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Q2, Q36, Q42, Q46, Q53, Q59, Q69, Q71, Q82, Q83, Q85, Q87, Q91, Q92</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+          <t>P4, P5, P35, P42, P46, P65, P66, P72, P75, Q3, Q5, Q7, Q22, Q23, Q49, Q63, Q69, Q71</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>31</v>
       </c>
       <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -25459,35 +25464,38 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>turvallinen / turvallisesti / turvallisuus</t>
+          <t>varmistaa / varmistua / huolehtia</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>safe / safely / safety</t>
+          <t>make sure / ensure / take care</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Usually points to the driver checking safety, destination, seat belt use, assisted handover, or customer comfort.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Q86 has several safety-sounding options; source chooses dispatch help</t>
+          <t>Not enough by itself if the option asks the driver to do something illegal, unsafe, or beyond the taxi-driver role.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Q6, Q74, Q83, Q86, Q87, Q91, Q92</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+          <t>P9, P20, P29, P33, P39, Q34, Q36, Q46, Q53, Q59, Q69, Q71, Q79, Q82, Q88, Q91, Q92, M27</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>24</v>
       </c>
       <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -25502,35 +25510,38 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>kysyä / tiedustella / tarvitseeko apua</t>
+          <t>kysyä / tiedustella / keskustella</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>ask / inquire / whether help is needed</t>
+          <t>ask / inquire / discuss / whether help is needed</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive when the driver asks before assisting, confirms wishes, route details, or a problem calmly.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Strong positive clue for disabled/visually impaired/slow-moving customers</t>
+          <t>If immediate emergency action is required, asking too much first may not be the best first step.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Q24, Q25, Q38, Q39, Q40, Q43, Q48, Q53, Q58, Q61, Q91, Q92</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+          <t>P26, P43, P74, Q25, Q48, Q52, Q58, Q75, Q92, M30, M37, M45, M47, M50, M60, M62, M73, M82</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>20</v>
       </c>
       <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -25545,35 +25556,38 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>sisälle / sisätilaan / turvallisesti sisällä</t>
+          <t>tarvittaessa auttaa / tarvittaessa avustaa / tarvittaessa</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>inside / indoors / safely inside</t>
+          <t>help/assist if necessary</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive when help is offered respectfully without forcing the passenger.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Correct clue when leaving child, night, care institution, or assisted customer</t>
+          <t>Do not assume every passenger needs help; ask or observe first unless the situation is clearly urgent.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Q2, Q46, Q87</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+          <t>P20, P29, P34, P40, Q34, Q45, Q51, Q56, Q71, Q91, M14, M24, M27, M43, M49, M51, M61</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>17</v>
       </c>
       <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -25588,35 +25602,38 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>poliisi / kutsun poliisin / soittaa poliisi</t>
+          <t>työnantaja / työnantajalta / selvität työnantajalta</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>police / call police</t>
+          <t>employer / check with employer</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive when authorization, work assignment, regular-taxi arrangement, or company process must be confirmed.</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Q83 is exception: source prefers refusing extremely drunk customer over automatically calling police</t>
+          <t>Driver responsibility for immediate safety cannot be handed to employer after the ride has already started.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Q7, Q22, Q23, Q49, Q63, Q69, Q71, Q77, Q83</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
+          <t>P4, P5, P26, P47, P53, P77, Q22, Q23, Q27, Q54, Q89, M40, M84, W5, W11, W33</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>16</v>
       </c>
       <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -25631,35 +25648,38 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Kela palvelunumero / tilausvälitysyhtiö / välityskeskus</t>
+          <t>kela / palvelunumero / tilausvälitysyhtiö</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Kela service number / dispatch</t>
+          <t>Kela / service number / dispatch company</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive when the driver cannot personally decide Kela entitlement, regular-taxi rights, or suitable vehicle arrangement.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Positive clue when driver cannot personally decide/arrange Kela or suitable vehicle alone</t>
+          <t>Do not replace official Kela/dispatch process with personal permission from the customer or guardian.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Q41, Q49</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>P30, P31, P32, P42, Q29, Q32, Q38, Q39, Q41, Q49, M28, M31, M34, M55</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>14</v>
       </c>
       <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -25674,35 +25694,38 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>työnantaja / selvitän työnantajalta / soitan työnantajalle</t>
+          <t>turvallinen / turvallisesti / turvallisuus</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>employer / check with employer / call employer</t>
+          <t>safe / safely / safety</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Strong positive clue when the answer protects the passenger, road users, or the driver.</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Positive clue when authorization or route problem is not the driver's solo decision</t>
+          <t>Check whether the option is practical and legal; a broad safety word can still be wrong if it ignores a specific rule.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Q22, Q23, Q27, Q54, Q89</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+          <t>P1, P3, P57, P63, P66, Q6, Q86, Q87, Q91, Q92, Q93, M12, W19, W22</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>14</v>
       </c>
       <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -25717,35 +25740,38 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>alkolukko + aina / estää käynnistyminen</t>
+          <t>alkolukko / asennettu alkolukko / estyy</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>alcohol interlock + always / prevents starting</t>
+          <t>alcohol interlock / installed / prevents starting</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive in school/day-care transport context where the vehicle must have an alcohol interlock.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Correct in school/day-care transport context</t>
+          <t>Not every taxi requires an alcohol interlock; the school/day-care transport context matters.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Q9, Q22, Q32, Q37, Q90</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+          <t>P4, P23, P54, P59, Q9, Q22, Q32, Q37, Q90, M20, M34, M78, W16</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>13</v>
       </c>
       <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -25760,35 +25786,38 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>asianmukainen / hyväksytty / sopiva</t>
+          <t>kohteliaasti / asiallisesti / rauhallisesti</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>appropriate / approved / suitable</t>
+          <t>politely / appropriately / calmly / kindly</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive in customer service, complaints, aggression, and passenger comfort situations.</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Strong positive safety-device clue</t>
+          <t>Politeness cannot override legal/safety duties such as seat belts, safe stopping, or accident response.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Q11, Q86, Q93, Q94, Q95</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+          <t>P36, P38, Q47, Q52, Q64, Q88, Q91, M50, M52, M53, M54, M59</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>12</v>
       </c>
       <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -25803,35 +25832,38 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>rungosta / neljästä pisteestä / jarrut päälle</t>
+          <t>oikeaan määränpäähän / määränpäähän / määränpäähän</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>by frame / four points / brakes on</t>
+          <t>right destination / sufficient language skill / communicate</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive when the driver’s duty is ensuring the customer reaches the correct destination safely.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Correct wheelchair securing clue</t>
+          <t>Sufficient language skill does not mean fluent conversation or same-language ability.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Q13, Q78</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>P9, P36, P63, P66, Q8, Q41, M1, M28, M53, M67, W19</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>11</v>
       </c>
       <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -25846,35 +25878,38 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>turvatyyny pois päältä</t>
+          <t>viipymättä / mahdollisimman pian / heti</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>airbag switched off</t>
+          <t>without delay / as soon as possible / immediately</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Usually positive for lost property, emergency response, safety reporting, and urgent assistance.</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Correct clue for rear-facing child seat in front</t>
+          <t>Time words are not enough if the action itself is wrong, such as abandoning a passenger quickly.</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Q19, Q80</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>P42, Q46, Q49, Q71, Q77, M44, M55, W1</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>8</v>
       </c>
       <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -25889,35 +25924,38 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>välttämätön</t>
+          <t>välttämätön / tarpeellinen / kuljetuksen suorittamiseksi välttämätön</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>necessary</t>
+          <t>necessary / necessary for carrying out the transport</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive for phone/hands-free or communication only when it is genuinely needed for the transport.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Correct clue for phone/hands-free communication only when needed for transport</t>
+          <t>Necessary does not permit speeding, unsafe stopping, or illegal customer requests.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Q16, Q18, Q20</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+          <t>P7, P11, Q18, Q20, M3, M6, M46, M76</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>8</v>
       </c>
       <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -25932,35 +25970,38 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>kohteliaasti / asiallisesti / rauhallisesti / ystävällisesti</t>
+          <t>handsfree / handsfree-laite / viestimet</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>politely / appropriately / calmly / kindly</t>
+          <t>hands-free / communication devices / making a call</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive only when communication is necessary and safe, especially with hands-free while driving.</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Positive service/de-escalation clue</t>
+          <t>Handheld phone use, messaging, or personal calls during transport are generally negative clues.</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Q47, Q52, Q64, Q88, Q91</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+          <t>P7, P11, P17, Q16, M3, M6, M8</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>7</v>
       </c>
       <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -25975,35 +26016,38 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>kuitti / kuitin tarjoaminen</t>
+          <t>sisälle / sisätilaan / kotiovesta sisään</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>receipt / offering a receipt</t>
+          <t>inside / indoors / received by staff/assistant</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive in questions about children, vulnerable customers, freezing weather, care institutions, or agreed assistants.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Source treats receipt offer as concrete taxi-service obligation</t>
+          <t>Do not expand this into medical/nursing tasks such as undressing or personal care unless specifically required and appropriate.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Q88</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>P29, P41, Q2, Q46, M16, M22, M44</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>7</v>
       </c>
       <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -26018,35 +26062,38 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>tarjota apua</t>
+          <t>asianmukainen / asianmukaisessa / hyväksytty</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>offer help</t>
+          <t>appropriate / approved / suitable</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive for child restraints, seat belts, vehicles, equipment, and safe customer transport.</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Positive when help is offered without forcing it</t>
+          <t>Still check the specific object: a suitable taxi or approved restraint is different from any improvised solution.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Q91</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>P12, Q11, Q86, Q93, Q94</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>P, Q</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -26061,35 +26108,38 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>omavastuu / enintään omavastuu</t>
+          <t>edullisin tarkoituksenmukainen reitti / tarkoituksenmukainen reitti / edullisin</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>deductible / at most deductible</t>
+          <t>most economical / appropriate route</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive when passenger leaves route choice to the driver or asks for route advice.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Correct Kela-payment clue</t>
+          <t>Do not blindly choose any route; customer preference and fairness matter.</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Q29</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>P51, M80, M99, M104, W9</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>5</v>
       </c>
       <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>P, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -26104,35 +26154,38 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>huoltaja / vanhempi / etukäteen</t>
+          <t>hengitysteiden avaaminen / hengitystiet / kylkiasento</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>guardian / parent / in advance</t>
+          <t>open airways / airways / recovery position / first aid</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive in first-aid and seizure/accident questions.</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Q27 and Q38 are exceptions: source uses employer/Kela entitlement rather than simple guardian/mother clue</t>
+          <t>Do not physically restrain convulsions or move an injured person unless necessary to save life/prevent further danger.</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Q27, Q42, Q44, Q87, Q95</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+          <t>P33, P68, Q36, M74, W24</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="I20" s="3" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -26147,35 +26200,38 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>asiakkaan kanssa / asiakkaalta / asiakas itse</t>
+          <t>opaskoira / työkoira / tunnistevaljaat</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>with/from the customer / customer themself</t>
+          <t>guide dog / working dog / identifying harness</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive in special-needs questions about guide dogs and working dogs.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Exception Q1/Q10: seat-belt responsibility depends on age/source framing</t>
+          <t>Do not distract, pet, or treat the guide dog as a normal pet during the job.</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Q31, Q45, Q48, Q50, Q51, Q58, Q85, Q92</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+          <t>P18, Q28, Q70, M29, M36</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>5</v>
       </c>
       <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -26190,35 +26246,38 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>pysäyttää ajoneuvo turvalliseen paikkaan</t>
+          <t>kuitti / kuitin tarjoaminen / annettava kuitti</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>stop vehicle in a safe place</t>
+          <t>receipt / offering or giving a receipt</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive because receipt must be offered/given after the ride/payment.</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Positive for customer conflict and first-aid situations</t>
+          <t>Receipt duty is separate from payment disputes; do not take a customer’s card or property by yourself.</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Q36</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>P80, Q88, M104, W47</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="I22" s="3" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -26233,35 +26292,38 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>koekäyttämällä</t>
+          <t>noudattaa / määräyksiä / liikenteen valvoja</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>by test-operating</t>
+          <t>obey/follow orders / traffic controller</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive when official traffic instructions override conflicting informal instructions.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Correct clue for accessible taxi lift inspection</t>
+          <t>Employer/customer instructions do not override police, traffic controller, or road rules.</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Q76</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>P5, Q5, Q23, M17</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>4</v>
       </c>
       <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -26276,35 +26338,38 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>ennakoida / toisen tienkäyttäjän toimintaa</t>
+          <t>rungosta / neljästä pisteestä / jarrut päälle</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>anticipate / other road user's actions</t>
+          <t>by frame / four points / brakes on</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Strong positive clue for securing a wheelchair safely in an accessible taxi.</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Correct road-user duty clue</t>
+          <t>Wheelchair brakes alone or normal seat belt alone are not enough for wheelchair securing.</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Q72</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>P14, P15, Q13, Q78</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>P, Q</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -26319,35 +26384,38 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>puuttua + ilmoittaa oppilaitokseen</t>
+          <t>ajopäiväkirja / ajopäiväkirja / työvuoron aloitus</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>intervene + report to school</t>
+          <t>driving logbook / shift start / break times</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Often signals the CORRECT answer</t>
+          <t>Positive in work-time and driving-logbook duty questions.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Correct clue for bullying during school transport</t>
+          <t>Do not include irrelevant personal details such as meals unless the law/company rule specifically asks.</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Q75, Q82</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>P64, M72, W20</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>3</v>
       </c>
       <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>P, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -26357,40 +26425,43 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>ei tarvitse</t>
+          <t>omavastuu / enintään omavastuu</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>does not need to</t>
+          <t>deductible / at most the deductible</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Positive in Kela-ride payment questions.</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Q81: phrase is in the question; do not automatically choose an option only because of it</t>
+          <t>Only applies when the ride is properly ordered as a Kela ride through the correct process.</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Q1, Q10, Q12, Q13, Q20, Q30, Q66, Q78, Q79, Q81, Q82</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+          <t>P31, Q29, M31</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="I26" s="3" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -26400,40 +26471,43 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>ilman</t>
+          <t>koekäyttämällä / koekäyttää / henkilönostin</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>without</t>
+          <t>test-operating / passenger lift</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Positive for accessible-taxi pre-departure equipment checks.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Usually wrong when it removes a safety device/permission; check context</t>
+          <t>A visual check alone may be too weak if the question asks how to check the lift.</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Q11, Q19, Q20, Q45, Q51, Q56, Q63, Q67, Q70, Q71, Q73, Q76, Q79, Q86, Q89</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+          <t>Q76, M4</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -26443,40 +26517,43 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>vain / ainoastaan</t>
+          <t>turvatyyny pois päältä / turvatyyny / airbag</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>only</t>
+          <t>airbag switched off</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Positive clue for rear-facing child restraint on the front passenger seat.</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Q29 uses 'enintään' not 'vain' and is correct; Q52 has customer choosing topic as correct</t>
+          <t>Airbag clue is context-specific; it does not remove normal child-restraint and seat-belt duties.</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Q15, Q19, Q31, Q38, Q52, Q53, Q60, Q61, Q68, Q72, Q76, Q78, Q84, Q89</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+          <t>Q19, Q80</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="I28" s="3" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -26486,40 +26563,43 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>ei koskaan / ei missään / ei voi koskaan</t>
+          <t>vastuullinen / roolimalli / esimerkillinen</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>never / in no situation</t>
+          <t>responsible / role model / exemplary</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Positive in school/day-care transport and general professional behaviour.</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>No strong exception in this set; it is usually too absolute</t>
+          <t>Being friendly or role-model-like still does not mean doing parent/school duties outside the driver role.</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Q19, Q51, Q61, Q80</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+          <t>P21</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -26534,35 +26614,38 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>asiakas päättää / oikeus valita</t>
+          <t>aina / aina silloin</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>customer decides / right to choose</t>
+          <t>always</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Can be suspicious because it may make an option too absolute.</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Q45 and Q52 are exceptions because customer independence/topic choice is positive</t>
+          <t>Often correct where the rule truly is absolute in that context, such as always using proper alkolukko in school/day-care transport or always offering receipt.</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Q6, Q13, Q52</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+          <t>P1, P6, P8, P10, P18, P27, P29, P34, P36, P39, P50, P52, P54, P59, P76, Q1, Q9, Q10</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>56</v>
       </c>
       <c r="I30" s="3" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -26577,35 +26660,38 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>ei kuljettajan vastuulla / asiakas vastuussa</t>
+          <t>vain / ainoastaan</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>not driver's responsibility / customer responsible</t>
+          <t>only</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Often too narrow when it limits a duty too much, such as only front seat, only customer service, only visual check.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Q95: parent/guardian is responsible for own child restraint</t>
+          <t>Can be correct in questions about strict legal limits or defined exceptions.</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Q59, Q62, Q66</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+          <t>P4, P13, P27, P30, P38, P47, P54, P55, P74, P78, P79, Q15, Q19, Q31, Q38, Q52, Q53, Q60</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>48</v>
       </c>
       <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -26620,35 +26706,38 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>lyhyt / alle minuutti / alle kilometri</t>
+          <t>ilman / kiinnittämättä / maksamatta</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>short / under a minute / under a kilometre</t>
+          <t>without / without doing</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Often negative when it means without seat belt, restraint, hands-free, payment, checking, or permission.</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>No safe shortcut exception; short trip/time usually does not remove duty</t>
+          <t>Can be neutral as context, for example “without advance booking”; do not judge this word alone.</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Q13, Q20, Q62, Q79, Q84</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+          <t>P6, P10, P12, P23, P39, P40, P50, P54, P78, Q7, Q11, Q19, Q20, Q37, Q45, Q51, Q56, Q63</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>42</v>
       </c>
       <c r="I32" s="3" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -26663,35 +26752,38 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>poikkeus / poikkeusajo</t>
+          <t>ei tarvitse / ei tarvi / tarvitse käyttää</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>exception / exceptional driving</t>
+          <t>does not need to</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Often wrong when it removes a safety, seat-belt, equipment, or service duty.</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Access exceptions can exist in traffic signs, but not as a general excuse</t>
+          <t>Can be correct when the law truly gives no duty in that exact context, so check who is responsible and the question wording.</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Q8, Q9, Q23, Q56</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+          <t>P8, P11, P13, P14, P22, P39, P51, P52, P71, Q1, Q10, Q12, Q13, Q20, Q30, Q66, Q78, Q79</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>30</v>
       </c>
       <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -26706,35 +26798,38 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>jos asiakas pyytää</t>
+          <t>kiire / kiireinen / myöhässä</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>if customer asks</t>
+          <t>hurry / busy / late / delay</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Negative if used to justify speeding, unsafe stopping, or breaking traffic rules.</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Q53: helping when the customer asks for comfort help is correct</t>
+          <t>Positive answer usually explains the delay, chooses the fastest legal route, and keeps the customer updated.</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Q6, Q15, Q17, Q57</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+          <t>P1, P24, P66, Q15, Q24, Q54, M11, M39, M94, W22, W37</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>11</v>
       </c>
       <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -26749,35 +26844,38 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>ei mukana avustaja / vaatii avustajan</t>
+          <t>jos asiakas pyytää / asiakas pyytää / pyytää ajamaan ylinopeutta</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>no assistant / requires assistant</t>
+          <t>if customer asks</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Customer request never permits speeding, unsafe stopping, illegal purchase, or abandoning safety duties.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>No exception: disability does not mean refusing the ride</t>
+          <t>Customer request can be valid for normal preferences, route selection, seat choice, or assistance style.</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Q40, Q43</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>P3, P37, P60, Q6, Q15, Q57, M11, M12, M64, M81</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>10</v>
       </c>
       <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -26792,35 +26890,38 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>odottaa autossa / ei tarvitse poistua</t>
+          <t>ei koskaan / missään tilanteessa / voi koskaan</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>wait in car / no need to leave car</t>
+          <t>never / in no situation</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Often too absolute and therefore wrong.</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>No strong exception in assisted-customer questions</t>
+          <t>Can be correct for clearly prohibited behaviour, such as handheld phone use or illegal alcohol-purchase requests.</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Q28, Q40, Q66</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+          <t>P40, Q19, Q51, Q61, Q66, Q80, M49, M91, W44</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>9</v>
       </c>
       <c r="I36" s="3" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -26835,35 +26936,38 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>ottaa maksukortti / ottaa käsilaukku itselle</t>
+          <t>ilman turvalaitetta / turvalaitetta ei / turvalaite ei</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>take payment card / keep handbag</t>
+          <t>without safety restraint/device</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Usually negative for children and accessibility safety.</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>No exception: do not take customer property</t>
+          <t>Taxi child-seat exceptions are narrow; under-3 and under-135 contexts need careful rule checking.</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Q7</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>P6, P10, P12, P50, Q11, Q67, Q79, M89, W43</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>9</v>
       </c>
       <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -26878,35 +26982,38 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>estää fyysisesti / huutaa / vastaa aggressioon</t>
+          <t>poikkeus / poikkeusajo / poikkeustapauksessa</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>physically stop / shout / answer aggression</t>
+          <t>exception / exceptional driving</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Often suspicious when used to justify bypassing alkolukko, stopping rules, or phone rules.</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>No exception: use calm/legal help instead</t>
+          <t>Some legal exceptions exist, but they must be explicitly stated and not invented by the driver.</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Q63, Q64, Q75</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+          <t>P2, P5, Q8, Q9, Q23, Q56, M1, M20, M61</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>9</v>
       </c>
       <c r="I38" s="3" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -26921,35 +27028,38 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>jätät / hylkäät / jätät huomiotta</t>
+          <t>jättää / hylkää / jätät huomiotta</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>leave / abandon / ignore</t>
+          <t>leave / abandon / ignore / continue normally</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Negative when safety, child, special-needs, accident, or lost-property duty exists.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>No exception when safety or child/special-customer duty exists</t>
+          <t>Can be correct only after you have ensured the customer/property/situation is safely handled.</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Q2, Q54, Q56, Q71, Q75, Q76, Q77</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+          <t>P33, P51, Q56, Q87, M22, M61, M99, W9</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>8</v>
       </c>
       <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -26964,35 +27074,38 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>ilman turvalaitetta</t>
+          <t>vapaaehtoista / vapaaehtoinen</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>without a safety restraint</t>
+          <t>voluntary / optional</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Usually wrong for seat belt, receipt, and mandatory driver duties.</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Q67 asks if child restraint is unavailable, but answer still uses back seat + seat belt</t>
+          <t>Some customer choices are voluntary, but legal safety and service duties are not.</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Q11, Q67, Q79, Q86</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+          <t>P8, P52, Q1, Q10, Q61, M18, W10, W47</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>8</v>
       </c>
       <c r="I40" s="3" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -27007,35 +27120,38 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>tarkastamatta / vain silmämääräisesti</t>
+          <t>ylinopeus / ylinopeutta / ylittää nopeusrajoitus</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>without checking / visual check only</t>
+          <t>speeding / exceed speed limit / speeding fines</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Strong negative clue: hurry or customer promise to pay fines never allows speeding.</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>No exception in lift/equipment check question</t>
+          <t>Emergency vehicles/legal emergency rules do not apply to ordinary taxi rides.</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Q76</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>P3, P66, Q15, Q54, M11, W22, W37</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>7</v>
       </c>
       <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -27050,35 +27166,38 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>ylinopeus / ylittää nopeusrajoitus</t>
+          <t>asiakas päättää / oikeus valita / saa valita pysähtymispaikan</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>speeding / exceed speed limit</t>
+          <t>customer decides / right to choose</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Often signals a WRONG answer</t>
+          <t>Negative when customer choice conflicts with safety, law, route fairness, payment rules, or driver responsibility.</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>No exception from customer request or schedule pressure</t>
+          <t>Customer can choose or influence the route when legal and fair; driver may still need to advise.</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Q15, Q54</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>P1, P14, P15, Q6, Q13, M12</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>6</v>
       </c>
       <c r="I42" s="3" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>P, Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -27088,32 +27207,43 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>mikä</t>
+          <t>lyhyt / alle minuutti / alle kilometri</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>what / which</t>
+          <t>short / under a minute / under a kilometre</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>asks for the correct thing or option</t>
+          <t>Usually wrong when it says a short distance/time removes safety or equipment duties.</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Mikä seuraavista on oikein? =&gt; Which of the following is correct?</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
+          <t>Short distance may matter only if the law or question explicitly sets that exception.</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>P14, P64, Q13, Q20, Q62, Q79</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>6</v>
+      </c>
       <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>P, Q</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -27123,32 +27253,43 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>mitä</t>
+          <t>takapenkillä ei tarvitse / kuljettajan ei tarvitse käyttää turvavyötä / ei tarvitse käyttää turvavyötä</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>what</t>
+          <t>back-seat/driver does not need seat belt</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>asks what you do or what something means</t>
+          <t>Usually negative: driver and passengers must follow seat-belt rules.</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Mitä sinun tulee tehdä? =&gt; What should you do?</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr"/>
-      <c r="H44" s="3" t="inlineStr"/>
+          <t>Responsibility for a 15+ passenger may be the passenger’s, but that does not make seat-belt use optional.</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>P22, Q30, Q81, M35, M102, W46</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>6</v>
+      </c>
       <c r="I44" s="3" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>P, Q, M, W</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -27158,32 +27299,43 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>kuka</t>
+          <t>henkilökohtaisia puheluita / lähettää viestejä / katsella televisiokuvaa</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>who</t>
+          <t>personal calls / send messages / watch screen</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>asks the person</t>
+          <t>Negative while driving or with customer on board.</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Kuka vastaa? =&gt; Who is responsible?</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr"/>
-      <c r="H45" s="4" t="inlineStr"/>
+          <t>Work-related communication may be allowed only if necessary and handled safely.</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>P7, P11, M6</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>P, M</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -27193,32 +27345,43 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>kenen</t>
+          <t>käsipuhelin / puhelin kädessä / pitää puhelinta kädessä</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>whose / who is responsible</t>
+          <t>handheld phone / phone in hand / without hands-free</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>very important for responsibility questions</t>
+          <t>Negative while driving; communication should be hands-free and only when necessary.</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Kenen vastuulla on? =&gt; Whose responsibility is it?</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="inlineStr"/>
-      <c r="H46" s="3" t="inlineStr"/>
+          <t>If stopped safely and legally, communication may be handled differently.</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>M3, M69, W39</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="I46" s="3" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>M, W</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -27228,32 +27391,43 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>kenellä</t>
+          <t>väkisin / fyysisesti / huutaa</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>who has / with whom</t>
+          <t>by force / physically / shout / push / hold tightly</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>asks who has authority, right, or responsibility</t>
+          <t>Negative in aggression, assistance, disability, and seizure situations.</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Kenellä on määräysvalta? =&gt; Who has authority?</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr"/>
-      <c r="H47" s="4" t="inlineStr"/>
+          <t>Physical action is only for immediate safety/first aid and must be proportionate; do not restrain convulsions.</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>P33, P35, Q63</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>P, Q</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -27263,32 +27437,43 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>missä</t>
+          <t>ei alkolukkoa / ilman alkolukkoa / olla käyttämättä alkolukkoa</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>where / in which</t>
+          <t>no alcohol interlock / without interlock / switch vehicle</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>place or situation</t>
+          <t>Negative in school/day-care transport where an alcohol interlock is required.</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Missä tilanteessa? =&gt; In which situation?</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr"/>
-      <c r="H48" s="3" t="inlineStr"/>
+          <t>Not every taxi needs alkolukko, so this clue depends on the transport type.</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Q9, M20</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -27298,32 +27483,43 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>mistä</t>
+          <t>huoltajan lupa / huoltajan valtuutus / kirjallinen lupa</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>from where / from what</t>
+          <t>guardian permission / authorisation</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>source, cause, or recognition clue</t>
+          <t>Suspicious when used to override child seat-belt duties or official Kela/regular-taxi processes.</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Mistä tunnistat? =&gt; How/from what do you recognise?</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr"/>
-      <c r="H49" s="4" t="inlineStr"/>
+          <t>Guardian involvement can be relevant for a child travelling alone, but it does not cancel legal safety duties.</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>Q27, M40</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -27333,32 +27529,43 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>mihin</t>
+          <t>kirjallinen valtakirja / valtakirja</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>to where / until what / for what</t>
+          <t>written power of attorney</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>destination, limit, or purpose</t>
+          <t>Often negative when it is used to justify buying alcohol or bypassing a formal process.</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Mihin asti? =&gt; Until what point/age?</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr"/>
-      <c r="H50" s="3" t="inlineStr"/>
+          <t>A written authorisation may matter in other legal contexts, but not for illegal or unsafe requests.</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Q57, M64</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="I50" s="3" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -27368,32 +27575,43 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>milloin</t>
+          <t>odottaa autossa / odotan autossa / ei tarvitse poistua</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>when</t>
+          <t>wait in car / no need to leave car</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>time or situation</t>
+          <t>Often wrong in assistance, slow passenger, visually impaired, wheelchair, or safe-exit questions.</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Milloin saat pysähtyä? =&gt; When may you stop?</t>
-        </is>
-      </c>
-      <c r="G51" s="4" t="inlineStr"/>
-      <c r="H51" s="4" t="inlineStr"/>
+          <t>May be acceptable when no help is needed and leaving the vehicle would create a safety problem.</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>Q66, M27</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -27403,32 +27621,43 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>miksi</t>
+          <t>tarkastamatta / silmämääräisesti / vain silmämääräisesti</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>why</t>
+          <t>without checking / visually only</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>reason</t>
+          <t>Negative in passenger-lift or equipment check questions.</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Miksi alkolukko vaaditaan? =&gt; Why is an alcohol interlock required?</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr"/>
-      <c r="H52" s="3" t="inlineStr"/>
+          <t>A visual check can be part of inspection, but not enough if functional testing is required.</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Q76, M4</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="I52" s="3" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Q, M</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -27438,32 +27667,43 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>miten</t>
+          <t>vain asiakaspalveluun / keskittyä vain asiakaspalveluun / vain omaan ajoneuvoon</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>how</t>
+          <t>only customer service / focus only on one thing</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>action or method</t>
+          <t>Wrong when it ignores traffic safety, anticipation, or special passenger needs.</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Miten toimit? =&gt; How do you act?</t>
-        </is>
-      </c>
-      <c r="G53" s="4" t="inlineStr"/>
-      <c r="H53" s="4" t="inlineStr"/>
+          <t>Customer service is important but never replaces legal and safety duties.</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>Q72, W48</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="I53" s="4" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Q, W</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -27473,32 +27713,43 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>kuinka</t>
+          <t>ei kuljettajan vastuulla / vastuu päättyy / ei ole sinun vastuullasi</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>how / how much / how long</t>
+          <t>not driver responsibility / responsibility ends / customer responsible</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>amount, duration, or method</t>
+          <t>Often negative when it tries to remove the driver’s duty to assist or ensure safety.</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>Kuinka kauan? =&gt; How long?</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr"/>
-      <c r="H54" s="3" t="inlineStr"/>
+          <t>Can be correct for 15+ seat-belt responsibility, but driver still manages safe transport.</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>P29</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="I54" s="3" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -27508,32 +27759,43 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>paljonko</t>
+          <t>oman harkinnan mukaan / minkä hyvänsä / minkä hyvänsä</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>how much</t>
+          <t>at own discretion / any route / anything</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>price or amount</t>
+          <t>Often wrong when it ignores rules, passenger interest, route fairness, or legal limits.</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>Paljonko asiakas maksaa? =&gt; How much does the customer pay?</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr"/>
-      <c r="H55" s="4" t="inlineStr"/>
+          <t>Driver judgement matters only within legal and professional boundaries.</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I55" s="4" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -27543,32 +27805,43 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>kauanko / kuinka kauan</t>
+          <t>ottaa maksukortti / lompakko / pantiksi</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>how long</t>
+          <t>take payment card/wallet/property as security</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>duration</t>
+          <t>Strong negative clue: driver should not take payment card, wallet, or valuables by force.</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Kuinka kauan ajolupa on voimassa? =&gt; How long is the permit valid?</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr"/>
-      <c r="H56" s="3" t="inlineStr"/>
+          <t>Use proper payment handling, discussion, dispatch/company process, or police if necessary.</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>P35</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="I56" s="3" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -27578,32 +27851,43 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>kumpi</t>
+          <t>soittaa torvea / rapsuttaa / napsuttaa</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>which of two</t>
+          <t>honk horn / pet/pat guide dog</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>choose between two</t>
+          <t>Negative in visually impaired/guide-dog service questions.</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Kumpi on oikein? =&gt; Which one is correct?</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr"/>
-      <c r="H57" s="4" t="inlineStr"/>
+          <t>Guide dog may ride with the customer, but should not be distracted.</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I57" s="4" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -27613,1070 +27897,34 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>WH-word</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>millainen</t>
+          <t>vaatii avustajan / ei mukana avustaja / avustaja ei ole mukana</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>what kind of</t>
+          <t>requires assistant / no assistant</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>asks description/type</t>
+          <t>Negative when it assumes disability means refusing service or requiring an assistant.</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Millainen toimintatapa? =&gt; What kind of way of acting?</t>
+          <t>If an agreed receiver/assistant is missing for a vulnerable person, wait or arrange safe handover.</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr"/>
-      <c r="H58" s="3" t="inlineStr"/>
+      <c r="H58" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="I58" s="3" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>CL056</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>WH-word</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>millä tavoin</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>in what way / how</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>asks method of action</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>Millä tavoin kuljettajan tulee toimia? =&gt; In what way should the driver act?</t>
-        </is>
-      </c>
-      <c r="G59" s="4" t="inlineStr"/>
-      <c r="H59" s="4" t="inlineStr"/>
-      <c r="I59" s="4" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>CL057</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>and</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>both connected ideas may matter</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>asiakas ja kuljettaja =&gt; customer and driver</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="inlineStr"/>
-      <c r="H60" s="3" t="inlineStr"/>
-      <c r="I60" s="3" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>CL058</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>sekä</t>
-        </is>
-      </c>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>and / as well as</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>formal 'and'; both parts matter</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>turvallisesti sekä kohteliaasti =&gt; safely and politely</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr"/>
-      <c r="H61" s="4" t="inlineStr"/>
-      <c r="I61" s="4" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>CL059</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>tai</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>or</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>one or the other</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>turvavyö tai turvalaite =&gt; seat belt or child restraint</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="inlineStr"/>
-      <c r="H62" s="3" t="inlineStr"/>
-      <c r="I62" s="3" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
-          <t>CL060</t>
-        </is>
-      </c>
-      <c r="B63" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>mutta</t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>but</t>
-        </is>
-      </c>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>contrast; after this word meaning may change</t>
-        </is>
-      </c>
-      <c r="F63" s="4" t="inlineStr">
-        <is>
-          <t>Kyllä, mutta vain... =&gt; Yes, but only...</t>
-        </is>
-      </c>
-      <c r="G63" s="4" t="inlineStr"/>
-      <c r="H63" s="4" t="inlineStr"/>
-      <c r="I63" s="4" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>CL061</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>koska</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>because</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>koska kuljettaja vastaa turvallisuudesta =&gt; because the driver is responsible for safety</t>
-        </is>
-      </c>
-      <c r="G64" s="3" t="inlineStr"/>
-      <c r="H64" s="3" t="inlineStr"/>
-      <c r="I64" s="3" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="4" t="inlineStr">
-        <is>
-          <t>CL062</t>
-        </is>
-      </c>
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>sillä</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>because / for</t>
-        </is>
-      </c>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>reason/explanation; similar to koska</t>
-        </is>
-      </c>
-      <c r="F65" s="4" t="inlineStr">
-        <is>
-          <t>sillä laki vaatii =&gt; because the law requires it</t>
-        </is>
-      </c>
-      <c r="G65" s="4" t="inlineStr"/>
-      <c r="H65" s="4" t="inlineStr"/>
-      <c r="I65" s="4" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>CL063</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>jotta</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>so that / in order to</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>purpose</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>jotta asiakas pääsee turvallisesti sisälle =&gt; so that the customer gets safely inside</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr"/>
-      <c r="H66" s="3" t="inlineStr"/>
-      <c r="I66" s="3" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>CL064</t>
-        </is>
-      </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>että</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>that</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>introduces content/explanation</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>varmistan, että asiakas pääsee sisälle =&gt; I make sure that the customer gets inside</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr"/>
-      <c r="H67" s="4" t="inlineStr"/>
-      <c r="I67" s="4" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>CL065</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>jos</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>if</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>jos asiakas pyytää =&gt; if the customer asks</t>
-        </is>
-      </c>
-      <c r="G68" s="3" t="inlineStr"/>
-      <c r="H68" s="3" t="inlineStr"/>
-      <c r="I68" s="3" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="inlineStr">
-        <is>
-          <t>CL066</t>
-        </is>
-      </c>
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>mikäli</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>if / provided that</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>formal if; common in exam wording</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>mikäli hän ei käytä turvavyötä =&gt; if they do not use the seat belt</t>
-        </is>
-      </c>
-      <c r="G69" s="4" t="inlineStr"/>
-      <c r="H69" s="4" t="inlineStr"/>
-      <c r="I69" s="4" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
-        <is>
-          <t>CL067</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>kun</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
-        <is>
-          <t>when</t>
-        </is>
-      </c>
-      <c r="E70" s="3" t="inlineStr">
-        <is>
-          <t>time/situation</t>
-        </is>
-      </c>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
-          <t>kun asiakas tulee kyytiin =&gt; when the customer gets in</t>
-        </is>
-      </c>
-      <c r="G70" s="3" t="inlineStr"/>
-      <c r="H70" s="3" t="inlineStr"/>
-      <c r="I70" s="3" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>CL068</t>
-        </is>
-      </c>
-      <c r="B71" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>kunnes</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="inlineStr">
-        <is>
-          <t>until</t>
-        </is>
-      </c>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>action continues until something happens</t>
-        </is>
-      </c>
-      <c r="F71" s="4" t="inlineStr">
-        <is>
-          <t>odotat kunnes avustaja saapuu =&gt; wait until the assistant arrives</t>
-        </is>
-      </c>
-      <c r="G71" s="4" t="inlineStr"/>
-      <c r="H71" s="4" t="inlineStr"/>
-      <c r="I71" s="4" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>CL069</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="inlineStr">
-        <is>
-          <t>vaikka</t>
-        </is>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>although / even if</t>
-        </is>
-      </c>
-      <c r="E72" s="3" t="inlineStr">
-        <is>
-          <t>contrast or exception</t>
-        </is>
-      </c>
-      <c r="F72" s="3" t="inlineStr">
-        <is>
-          <t>vaikka asiakas pyytää =&gt; even if the customer asks</t>
-        </is>
-      </c>
-      <c r="G72" s="3" t="inlineStr"/>
-      <c r="H72" s="3" t="inlineStr"/>
-      <c r="I72" s="3" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>CL070</t>
-        </is>
-      </c>
-      <c r="B73" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>ellei</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>unless / if not</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>negative condition; very important</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>ellei huoltaja ole mukana =&gt; if/unless the guardian is not present</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="inlineStr"/>
-      <c r="H73" s="4" t="inlineStr"/>
-      <c r="I73" s="4" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="3" t="inlineStr">
-        <is>
-          <t>CL071</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C74" s="3" t="inlineStr">
-        <is>
-          <t>ennen kuin</t>
-        </is>
-      </c>
-      <c r="D74" s="3" t="inlineStr">
-        <is>
-          <t>before</t>
-        </is>
-      </c>
-      <c r="E74" s="3" t="inlineStr">
-        <is>
-          <t>order of action</t>
-        </is>
-      </c>
-      <c r="F74" s="3" t="inlineStr">
-        <is>
-          <t>ennen kuin matka alkaa =&gt; before the trip starts</t>
-        </is>
-      </c>
-      <c r="G74" s="3" t="inlineStr"/>
-      <c r="H74" s="3" t="inlineStr"/>
-      <c r="I74" s="3" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>CL072</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>sen jälkeen kun</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>after</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>after something happens</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>sen jälkeen kun asiakas poistuu =&gt; after the customer exits</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr"/>
-      <c r="H75" s="4" t="inlineStr"/>
-      <c r="I75" s="4" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="3" t="inlineStr">
-        <is>
-          <t>CL073</t>
-        </is>
-      </c>
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t>silloin kun</t>
-        </is>
-      </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>when / in the situation where</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="inlineStr">
-        <is>
-          <t>specific condition</t>
-        </is>
-      </c>
-      <c r="F76" s="3" t="inlineStr">
-        <is>
-          <t>silloin kun asiakas matkustaa yksin =&gt; when the customer travels alone</t>
-        </is>
-      </c>
-      <c r="G76" s="3" t="inlineStr"/>
-      <c r="H76" s="3" t="inlineStr"/>
-      <c r="I76" s="3" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>CL074</t>
-        </is>
-      </c>
-      <c r="B77" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>sekä</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>as well as</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr"/>
-      <c r="F77" s="4" t="inlineStr"/>
-      <c r="G77" s="4" t="inlineStr"/>
-      <c r="H77" s="4" t="inlineStr"/>
-      <c r="I77" s="4" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="3" t="inlineStr">
-        <is>
-          <t>CL075</t>
-        </is>
-      </c>
-      <c r="B78" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C78" s="3" t="inlineStr">
-        <is>
-          <t>siten että</t>
-        </is>
-      </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>so that / in such a way that</t>
-        </is>
-      </c>
-      <c r="E78" s="3" t="inlineStr">
-        <is>
-          <t>method/result</t>
-        </is>
-      </c>
-      <c r="F78" s="3" t="inlineStr">
-        <is>
-          <t>kiinnitetään siten, että se ei liiku =&gt; secured so that it does not move</t>
-        </is>
-      </c>
-      <c r="G78" s="3" t="inlineStr"/>
-      <c r="H78" s="3" t="inlineStr"/>
-      <c r="I78" s="3" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="4" t="inlineStr">
-        <is>
-          <t>CL076</t>
-        </is>
-      </c>
-      <c r="B79" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>kuitenkin</t>
-        </is>
-      </c>
-      <c r="D79" s="4" t="inlineStr">
-        <is>
-          <t>however</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>exception/contrast</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>kuitenkin kuljettaja vastaa =&gt; however, the driver is responsible</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr"/>
-      <c r="H79" s="4" t="inlineStr"/>
-      <c r="I79" s="4" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="3" t="inlineStr">
-        <is>
-          <t>CL077</t>
-        </is>
-      </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C80" s="3" t="inlineStr">
-        <is>
-          <t>myös</t>
-        </is>
-      </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>also</t>
-        </is>
-      </c>
-      <c r="E80" s="3" t="inlineStr">
-        <is>
-          <t>additional point</t>
-        </is>
-      </c>
-      <c r="F80" s="3" t="inlineStr">
-        <is>
-          <t>kuljettajan tulee myös varmistaa =&gt; the driver must also make sure</t>
-        </is>
-      </c>
-      <c r="G80" s="3" t="inlineStr"/>
-      <c r="H80" s="3" t="inlineStr"/>
-      <c r="I80" s="3" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="4" t="inlineStr">
-        <is>
-          <t>CL078</t>
-        </is>
-      </c>
-      <c r="B81" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="inlineStr">
-        <is>
-          <t>vain</t>
-        </is>
-      </c>
-      <c r="D81" s="4" t="inlineStr">
-        <is>
-          <t>only</t>
-        </is>
-      </c>
-      <c r="E81" s="4" t="inlineStr">
-        <is>
-          <t>limiting word; often a trap</t>
-        </is>
-      </c>
-      <c r="F81" s="4" t="inlineStr">
-        <is>
-          <t>vain jos =&gt; only if</t>
-        </is>
-      </c>
-      <c r="G81" s="4" t="inlineStr"/>
-      <c r="H81" s="4" t="inlineStr"/>
-      <c r="I81" s="4" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
-        <is>
-          <t>CL079</t>
-        </is>
-      </c>
-      <c r="B82" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C82" s="3" t="inlineStr">
-        <is>
-          <t>aina</t>
-        </is>
-      </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>always</t>
-        </is>
-      </c>
-      <c r="E82" s="3" t="inlineStr">
-        <is>
-          <t>strong word; can be correct or dangerous</t>
-        </is>
-      </c>
-      <c r="F82" s="3" t="inlineStr">
-        <is>
-          <t>aina käyttää turvavyötä =&gt; always use a seat belt</t>
-        </is>
-      </c>
-      <c r="G82" s="3" t="inlineStr"/>
-      <c r="H82" s="3" t="inlineStr"/>
-      <c r="I82" s="3" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="4" t="inlineStr">
-        <is>
-          <t>CL080</t>
-        </is>
-      </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>ei koskaan</t>
-        </is>
-      </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>never</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>strong negative</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>ei koskaan saa =&gt; must never</t>
-        </is>
-      </c>
-      <c r="G83" s="4" t="inlineStr"/>
-      <c r="H83" s="4" t="inlineStr"/>
-      <c r="I83" s="4" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="3" t="inlineStr">
-        <is>
-          <t>CL081</t>
-        </is>
-      </c>
-      <c r="B84" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C84" s="3" t="inlineStr">
-        <is>
-          <t>tarvittaessa</t>
-        </is>
-      </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>if necessary / when needed</t>
-        </is>
-      </c>
-      <c r="E84" s="3" t="inlineStr">
-        <is>
-          <t>often correct in assistance questions</t>
-        </is>
-      </c>
-      <c r="F84" s="3" t="inlineStr">
-        <is>
-          <t>avustaa tarvittaessa =&gt; assist if necessary</t>
-        </is>
-      </c>
-      <c r="G84" s="3" t="inlineStr"/>
-      <c r="H84" s="3" t="inlineStr"/>
-      <c r="I84" s="3" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="4" t="inlineStr">
-        <is>
-          <t>CL082</t>
-        </is>
-      </c>
-      <c r="B85" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
-        <is>
-          <t>mahdollisimman pian</t>
-        </is>
-      </c>
-      <c r="D85" s="4" t="inlineStr">
-        <is>
-          <t>as soon as possible</t>
-        </is>
-      </c>
-      <c r="E85" s="4" t="inlineStr">
-        <is>
-          <t>often correct for lost property/safety</t>
-        </is>
-      </c>
-      <c r="F85" s="4" t="inlineStr">
-        <is>
-          <t>toimita mahdollisimman pian =&gt; deliver as soon as possible</t>
-        </is>
-      </c>
-      <c r="G85" s="4" t="inlineStr"/>
-      <c r="H85" s="4" t="inlineStr"/>
-      <c r="I85" s="4" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="3" t="inlineStr">
-        <is>
-          <t>CL083</t>
-        </is>
-      </c>
-      <c r="B86" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C86" s="3" t="inlineStr">
-        <is>
-          <t>viipymättä</t>
-        </is>
-      </c>
-      <c r="D86" s="3" t="inlineStr">
-        <is>
-          <t>without delay</t>
-        </is>
-      </c>
-      <c r="E86" s="3" t="inlineStr">
-        <is>
-          <t>strong correct clue</t>
-        </is>
-      </c>
-      <c r="F86" s="3" t="inlineStr">
-        <is>
-          <t>toimita viipymättä =&gt; deliver without delay</t>
-        </is>
-      </c>
-      <c r="G86" s="3" t="inlineStr"/>
-      <c r="H86" s="3" t="inlineStr"/>
-      <c r="I86" s="3" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="4" t="inlineStr">
-        <is>
-          <t>CL084</t>
-        </is>
-      </c>
-      <c r="B87" s="4" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C87" s="4" t="inlineStr">
-        <is>
-          <t>joka</t>
-        </is>
-      </c>
-      <c r="D87" s="4" t="inlineStr">
-        <is>
-          <t>who/which/what</t>
-        </is>
-      </c>
-      <c r="E87" s="4" t="inlineStr">
-        <is>
-          <t>refering previous word  jonka(whose),jota(whom),jossa(in which),josta(from which)</t>
-        </is>
-      </c>
-      <c r="F87" s="4" t="inlineStr"/>
-      <c r="G87" s="4" t="inlineStr"/>
-      <c r="H87" s="4" t="inlineStr"/>
-      <c r="I87" s="4" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="3" t="inlineStr">
-        <is>
-          <t>CL085</t>
-        </is>
-      </c>
-      <c r="B88" s="3" t="inlineStr">
-        <is>
-          <t>Conjunction</t>
-        </is>
-      </c>
-      <c r="C88" s="3" t="inlineStr">
-        <is>
-          <t>välittömästi</t>
-        </is>
-      </c>
-      <c r="D88" s="3" t="inlineStr">
-        <is>
-          <t>immediately</t>
-        </is>
-      </c>
-      <c r="E88" s="3" t="inlineStr">
-        <is>
-          <t>strong time clue</t>
-        </is>
-      </c>
-      <c r="F88" s="3" t="inlineStr">
-        <is>
-          <t>soita välittömästi =&gt; call immediately</t>
-        </is>
-      </c>
-      <c r="G88" s="3" t="inlineStr"/>
-      <c r="H88" s="3" t="inlineStr"/>
-      <c r="I88" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>